<commit_message>
Update Sprint 1 scrum workbook
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1.xlsx
+++ b/documentation/scrum/Sprint_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{973D76C4-0745-455A-BB68-1F9FD64BF1AA}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{692240A2-B13A-4ADC-BDE1-6B1DC5180EA4}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -305,9 +305,6 @@
     <t>Prepare Meeting 01 minutes</t>
   </si>
   <si>
-    <t>Meeting_01_Week_01.docx</t>
-  </si>
-  <si>
     <t>Upload to documentation/meetings</t>
   </si>
   <si>
@@ -375,6 +372,9 @@
   </si>
   <si>
     <t>What are the main priorities for Sprint 2?</t>
+  </si>
+  <si>
+    <t>Meeting_01.docx</t>
   </si>
 </sst>
 </file>
@@ -1292,21 +1292,21 @@
         <v>25</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>23</v>
@@ -1318,13 +1318,13 @@
         <v>25</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1351,7 +1351,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1359,74 +1359,74 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>

</xml_diff>

<commit_message>
Update meeting and sprint documentation
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1.xlsx
+++ b/documentation/scrum/Sprint_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{692240A2-B13A-4ADC-BDE1-6B1DC5180EA4}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CA4DFED-F420-46F3-80F0-E76C4EBD786A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint 1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="121">
   <si>
     <t>CIS4014-N Interactive Visualisation – Group 4 | Sprint 1 – Week 01</t>
   </si>
@@ -278,9 +278,6 @@
     <t>Initial dataset analysis</t>
   </si>
   <si>
-    <t>Imasha + Member 2</t>
-  </si>
-  <si>
     <t>Variable and data-quality notes</t>
   </si>
   <si>
@@ -375,6 +372,18 @@
   </si>
   <si>
     <t>Meeting_01.docx</t>
+  </si>
+  <si>
+    <t>Samarakoon</t>
+  </si>
+  <si>
+    <t>Ilamperuma</t>
+  </si>
+  <si>
+    <t>De Silva</t>
+  </si>
+  <si>
+    <t>Ilamperuma + Samarakoon + De Silva</t>
   </si>
 </sst>
 </file>
@@ -456,6 +465,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -765,7 +778,7 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="3" max="3" width="19.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="42" customWidth="1"/>
@@ -1075,7 +1088,7 @@
         <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>47</v>
+        <v>117</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>24</v>
@@ -1101,7 +1114,7 @@
         <v>63</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>52</v>
+        <v>118</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>24</v>
@@ -1127,7 +1140,7 @@
         <v>67</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>56</v>
+        <v>119</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>24</v>
@@ -1153,7 +1166,7 @@
         <v>71</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>24</v>
@@ -1179,7 +1192,7 @@
         <v>76</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>24</v>
@@ -1205,7 +1218,7 @@
         <v>80</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>38</v>
@@ -1223,7 +1236,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>83</v>
       </c>
@@ -1231,7 +1244,7 @@
         <v>84</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>24</v>
@@ -1240,24 +1253,24 @@
         <v>25</v>
       </c>
       <c r="F25" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="C26" s="2" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>24</v>
@@ -1266,24 +1279,24 @@
         <v>25</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="C27" s="2" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>38</v>
@@ -1292,24 +1305,24 @@
         <v>25</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="C28" s="2" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>38</v>
@@ -1318,13 +1331,13 @@
         <v>25</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1332,8 +1345,9 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1351,7 +1365,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A1" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1359,74 +1373,74 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>

</xml_diff>

<commit_message>
Add coffee sales data and update project documents
</commit_message>
<xml_diff>
--- a/documentation/scrum/Sprint_1.xlsx
+++ b/documentation/scrum/Sprint_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://micloud365-my.sharepoint.com/personal/imashai_millenniumitesp_com/Documents/Desktop/MSc BInA/Academics/3-Interactive Visualization/Assesment/Project/group4-interactive-visualisation/documentation/scrum/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CA4DFED-F420-46F3-80F0-E76C4EBD786A}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="11_4D63132A0E366EB0700ABEF92BB88AC76CF52F45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFEB0238-5332-4882-A9E0-35A2A050CB72}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -128,9 +128,6 @@
     <t>Selected dataset and source</t>
   </si>
   <si>
-    <t>Save dataset/source details</t>
-  </si>
-  <si>
     <t>S1-04</t>
   </si>
   <si>
@@ -245,9 +242,6 @@
     <t>Day 1–2</t>
   </si>
   <si>
-    <t>Screenshot board for evidence</t>
-  </si>
-  <si>
     <t>S1-13</t>
   </si>
   <si>
@@ -257,9 +251,6 @@
     <t>Shared GitHub repository</t>
   </si>
   <si>
-    <t>Record repository setup</t>
-  </si>
-  <si>
     <t>S1-14</t>
   </si>
   <si>
@@ -269,9 +260,6 @@
     <t>Project folders created</t>
   </si>
   <si>
-    <t>Commit structure to repository</t>
-  </si>
-  <si>
     <t>S1-15</t>
   </si>
   <si>
@@ -293,18 +281,12 @@
     <t>Master task list</t>
   </si>
   <si>
-    <t>Maintain in Trello</t>
-  </si>
-  <si>
     <t>S1-17</t>
   </si>
   <si>
     <t>Prepare Meeting 01 minutes</t>
   </si>
   <si>
-    <t>Upload to documentation/meetings</t>
-  </si>
-  <si>
     <t>S1-18</t>
   </si>
   <si>
@@ -384,13 +366,31 @@
   </si>
   <si>
     <t>Ilamperuma + Samarakoon + De Silva</t>
+  </si>
+  <si>
+    <t>https://trello.com/b/k5MT44Ww/group-4-cis4014-n-interactive-visualisation</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation</t>
+  </si>
+  <si>
+    <t>https://github.com/inkymello/group4-interactive-visualisation/blob/main/README_STRUCTURE.md</t>
+  </si>
+  <si>
+    <t>Uploaded to documentation/meetings to github</t>
+  </si>
+  <si>
+    <t>Maintained in Trello</t>
+  </si>
+  <si>
+    <t>Coffe Shop Sales Dataset</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,6 +413,14 @@
       <sz val="15"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -431,10 +439,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -442,6 +451,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -451,7 +463,8 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -465,10 +478,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -783,20 +792,20 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="42" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
+    <col min="8" max="8" width="85.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -947,41 +956,41 @@
         <v>4</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>23</v>
@@ -993,24 +1002,24 @@
         <v>25</v>
       </c>
       <c r="F15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>24</v>
@@ -1019,24 +1028,24 @@
         <v>25</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>24</v>
@@ -1045,24 +1054,24 @@
         <v>25</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>24</v>
@@ -1071,24 +1080,24 @@
         <v>25</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="C19" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>24</v>
@@ -1097,24 +1106,24 @@
         <v>25</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C20" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>24</v>
@@ -1123,24 +1132,24 @@
         <v>25</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="C21" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>24</v>
@@ -1149,24 +1158,24 @@
         <v>25</v>
       </c>
       <c r="F21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>24</v>
@@ -1175,24 +1184,24 @@
         <v>25</v>
       </c>
       <c r="F22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G22" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>74</v>
+      <c r="H22" s="4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>24</v>
@@ -1201,50 +1210,50 @@
         <v>25</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>25</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H24" s="2" t="s">
-        <v>82</v>
+      <c r="H24" s="4" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>24</v>
@@ -1253,24 +1262,24 @@
         <v>25</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>24</v>
@@ -1279,75 +1288,80 @@
         <v>25</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>4</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>90</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>25</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="H23" r:id="rId1" xr:uid="{CB1D5040-D46E-4C0B-AAB7-A892F284A20A}"/>
+    <hyperlink ref="H22" r:id="rId2" xr:uid="{018413AF-582F-47AF-8603-8D1ADC098FB5}"/>
+    <hyperlink ref="H24" r:id="rId3" xr:uid="{CF940C84-0815-44AA-A165-67100D26A0D4}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1364,83 +1378,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>

</xml_diff>